<commit_message>
jeu de données traits spécifiques propres sans extraction encore
</commit_message>
<xml_diff>
--- a/output/site_info_clean.xlsx
+++ b/output/site_info_clean.xlsx
@@ -351,7 +351,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:J929"/>
+  <dimension ref="A1:J953"/>
   <sheetFormatPr defaultRowHeight="15"/>
   <sheetData>
     <row r="1" s="1" customFormat="1">
@@ -14996,7 +14996,7 @@
       </c>
       <c r="B545" t="inlineStr">
         <is>
-          <t>Mesnil st père2</t>
+          <t>Mesnil st père 2</t>
         </is>
       </c>
       <c r="E545" t="inlineStr">
@@ -15016,7 +15016,7 @@
       </c>
       <c r="B546" t="inlineStr">
         <is>
-          <t>Mesnil st père2</t>
+          <t>Mesnil st père 2</t>
         </is>
       </c>
       <c r="E546" t="inlineStr">
@@ -15036,7 +15036,7 @@
       </c>
       <c r="B547" t="inlineStr">
         <is>
-          <t>Mesnil st père2</t>
+          <t>Mesnil st père 2</t>
         </is>
       </c>
       <c r="E547" t="inlineStr">
@@ -15056,7 +15056,7 @@
       </c>
       <c r="B548" t="inlineStr">
         <is>
-          <t>Mesnil st père2</t>
+          <t>Mesnil st père 2</t>
         </is>
       </c>
       <c r="E548" t="inlineStr">
@@ -15076,7 +15076,7 @@
       </c>
       <c r="B549" t="inlineStr">
         <is>
-          <t>Mesnil st père2</t>
+          <t>Mesnil st père 2</t>
         </is>
       </c>
       <c r="E549" t="inlineStr">
@@ -15096,7 +15096,7 @@
       </c>
       <c r="B550" t="inlineStr">
         <is>
-          <t>Mesnil st père2</t>
+          <t>Mesnil st père 2</t>
         </is>
       </c>
       <c r="E550" t="inlineStr">
@@ -15116,7 +15116,7 @@
       </c>
       <c r="B551" t="inlineStr">
         <is>
-          <t>Mesnil st père2</t>
+          <t>Mesnil st père 2</t>
         </is>
       </c>
       <c r="E551" t="inlineStr">
@@ -15136,7 +15136,7 @@
       </c>
       <c r="B552" t="inlineStr">
         <is>
-          <t>Mesnil st père2</t>
+          <t>Mesnil st père 2</t>
         </is>
       </c>
       <c r="E552" t="inlineStr">
@@ -15156,7 +15156,7 @@
       </c>
       <c r="B553" t="inlineStr">
         <is>
-          <t>Mesnil st père2</t>
+          <t>Mesnil st père 2</t>
         </is>
       </c>
       <c r="E553" t="inlineStr">
@@ -22261,7 +22261,7 @@
       </c>
       <c r="B819" t="inlineStr">
         <is>
-          <t>Gîte</t>
+          <t>Gite</t>
         </is>
       </c>
       <c r="C819" t="inlineStr">
@@ -22291,7 +22291,7 @@
       </c>
       <c r="B820" t="inlineStr">
         <is>
-          <t>Gîte</t>
+          <t>Gite</t>
         </is>
       </c>
       <c r="C820" t="inlineStr">
@@ -22316,7 +22316,7 @@
       </c>
       <c r="B821" t="inlineStr">
         <is>
-          <t>Gîte</t>
+          <t>Gite</t>
         </is>
       </c>
       <c r="C821" t="inlineStr">
@@ -22341,7 +22341,7 @@
       </c>
       <c r="B822" t="inlineStr">
         <is>
-          <t>Gîte</t>
+          <t>Gite</t>
         </is>
       </c>
       <c r="C822" t="inlineStr">
@@ -22366,7 +22366,7 @@
       </c>
       <c r="B823" t="inlineStr">
         <is>
-          <t>Gîte</t>
+          <t>Gite</t>
         </is>
       </c>
       <c r="C823" t="inlineStr">
@@ -22391,7 +22391,7 @@
       </c>
       <c r="B824" t="inlineStr">
         <is>
-          <t>Gîte</t>
+          <t>Gite</t>
         </is>
       </c>
       <c r="C824" t="inlineStr">
@@ -22416,7 +22416,7 @@
       </c>
       <c r="B825" t="inlineStr">
         <is>
-          <t>Gîte</t>
+          <t>Gite</t>
         </is>
       </c>
       <c r="F825" t="inlineStr">
@@ -22431,7 +22431,7 @@
       </c>
       <c r="B826" t="inlineStr">
         <is>
-          <t>Gîte</t>
+          <t>Gite</t>
         </is>
       </c>
       <c r="F826" t="inlineStr">
@@ -22446,7 +22446,7 @@
       </c>
       <c r="B827" t="inlineStr">
         <is>
-          <t>Gîte</t>
+          <t>Gite</t>
         </is>
       </c>
       <c r="F827" t="inlineStr">
@@ -22461,7 +22461,7 @@
       </c>
       <c r="B828" t="inlineStr">
         <is>
-          <t>Gîte</t>
+          <t>Gite</t>
         </is>
       </c>
       <c r="F828" t="inlineStr">
@@ -22476,7 +22476,7 @@
       </c>
       <c r="B829" t="inlineStr">
         <is>
-          <t>Gîte</t>
+          <t>Gite</t>
         </is>
       </c>
       <c r="F829" t="inlineStr">
@@ -22491,7 +22491,7 @@
       </c>
       <c r="B830" t="inlineStr">
         <is>
-          <t>Gîte</t>
+          <t>Gite</t>
         </is>
       </c>
       <c r="F830" t="inlineStr">
@@ -22506,7 +22506,7 @@
       </c>
       <c r="B831" t="inlineStr">
         <is>
-          <t>Gîte</t>
+          <t>Gite</t>
         </is>
       </c>
       <c r="F831" t="inlineStr">
@@ -24101,7 +24101,7 @@
       </c>
       <c r="B891" t="inlineStr">
         <is>
-          <t>Gîte</t>
+          <t>Gite</t>
         </is>
       </c>
       <c r="D891" t="inlineStr">
@@ -24126,7 +24126,7 @@
       </c>
       <c r="B892" t="inlineStr">
         <is>
-          <t>Gîte</t>
+          <t>Gite</t>
         </is>
       </c>
       <c r="D892" t="inlineStr">
@@ -24151,7 +24151,7 @@
       </c>
       <c r="B893" t="inlineStr">
         <is>
-          <t>Gîte</t>
+          <t>Gite</t>
         </is>
       </c>
       <c r="D893" t="inlineStr">
@@ -24176,7 +24176,7 @@
       </c>
       <c r="B894" t="inlineStr">
         <is>
-          <t>Gîte</t>
+          <t>Gite</t>
         </is>
       </c>
       <c r="D894" t="inlineStr">
@@ -24201,7 +24201,7 @@
       </c>
       <c r="B895" t="inlineStr">
         <is>
-          <t>Gîte</t>
+          <t>Gite</t>
         </is>
       </c>
       <c r="D895" t="inlineStr">
@@ -24226,7 +24226,7 @@
       </c>
       <c r="B896" t="inlineStr">
         <is>
-          <t>Gîte</t>
+          <t>Gite</t>
         </is>
       </c>
       <c r="D896" t="inlineStr">
@@ -24251,7 +24251,7 @@
       </c>
       <c r="B897" t="inlineStr">
         <is>
-          <t>Gîte</t>
+          <t>Gite</t>
         </is>
       </c>
       <c r="D897" t="inlineStr">
@@ -24276,7 +24276,7 @@
       </c>
       <c r="B898" t="inlineStr">
         <is>
-          <t>Gîte</t>
+          <t>Gite</t>
         </is>
       </c>
       <c r="E898" t="inlineStr">
@@ -24346,7 +24346,7 @@
       </c>
       <c r="B901" t="inlineStr">
         <is>
-          <t>Gîte</t>
+          <t>Gite</t>
         </is>
       </c>
       <c r="D901" t="inlineStr">
@@ -24371,7 +24371,7 @@
       </c>
       <c r="B902" t="inlineStr">
         <is>
-          <t>Gîte</t>
+          <t>Gite</t>
         </is>
       </c>
       <c r="D902" t="inlineStr">
@@ -24396,7 +24396,7 @@
       </c>
       <c r="B903" t="inlineStr">
         <is>
-          <t>Gîte</t>
+          <t>Gite</t>
         </is>
       </c>
       <c r="D903" t="inlineStr">
@@ -24421,7 +24421,7 @@
       </c>
       <c r="B904" t="inlineStr">
         <is>
-          <t>Gîte</t>
+          <t>Gite</t>
         </is>
       </c>
       <c r="D904" t="inlineStr">
@@ -24446,7 +24446,7 @@
       </c>
       <c r="B905" t="inlineStr">
         <is>
-          <t>Gîte</t>
+          <t>Gite</t>
         </is>
       </c>
       <c r="D905" t="inlineStr">
@@ -24479,6 +24479,11 @@
           <t>45</t>
         </is>
       </c>
+      <c r="E906" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
       <c r="F906" t="inlineStr">
         <is>
           <t>Reg</t>
@@ -24499,6 +24504,11 @@
           <t>40</t>
         </is>
       </c>
+      <c r="E907" t="inlineStr">
+        <is>
+          <t>30</t>
+        </is>
+      </c>
       <c r="F907" t="inlineStr">
         <is>
           <t>Reg</t>
@@ -24519,6 +24529,11 @@
           <t>100</t>
         </is>
       </c>
+      <c r="E908" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
       <c r="F908" t="inlineStr">
         <is>
           <t>Reg</t>
@@ -24564,6 +24579,11 @@
           <t>50</t>
         </is>
       </c>
+      <c r="E910" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
       <c r="F910" t="inlineStr">
         <is>
           <t>Reg</t>
@@ -24576,7 +24596,7 @@
       </c>
       <c r="B911" t="inlineStr">
         <is>
-          <t>Gîte</t>
+          <t>Gite</t>
         </is>
       </c>
       <c r="D911" t="inlineStr">
@@ -24709,6 +24729,11 @@
           <t>45</t>
         </is>
       </c>
+      <c r="E916" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
       <c r="F916" t="inlineStr">
         <is>
           <t>FP</t>
@@ -24729,6 +24754,11 @@
           <t>40</t>
         </is>
       </c>
+      <c r="E917" t="inlineStr">
+        <is>
+          <t>20</t>
+        </is>
+      </c>
       <c r="F917" t="inlineStr">
         <is>
           <t>FP</t>
@@ -24749,6 +24779,11 @@
           <t>50</t>
         </is>
       </c>
+      <c r="E918" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
       <c r="F918" t="inlineStr">
         <is>
           <t>FP</t>
@@ -24769,6 +24804,11 @@
           <t>50</t>
         </is>
       </c>
+      <c r="E919" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
       <c r="F919" t="inlineStr">
         <is>
           <t>FP</t>
@@ -25022,6 +25062,611 @@
       <c r="F929" t="inlineStr">
         <is>
           <t>FP</t>
+        </is>
+      </c>
+    </row>
+    <row r="930">
+      <c r="A930">
+        <v>2026</v>
+      </c>
+      <c r="B930" t="inlineStr">
+        <is>
+          <t>Mesnil st père</t>
+        </is>
+      </c>
+      <c r="D930" t="inlineStr">
+        <is>
+          <t>45</t>
+        </is>
+      </c>
+      <c r="E930" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+      <c r="F930" t="inlineStr">
+        <is>
+          <t>FT</t>
+        </is>
+      </c>
+    </row>
+    <row r="931">
+      <c r="A931">
+        <v>2026</v>
+      </c>
+      <c r="B931" t="inlineStr">
+        <is>
+          <t>Mesnil st père</t>
+        </is>
+      </c>
+      <c r="D931" t="inlineStr">
+        <is>
+          <t>55</t>
+        </is>
+      </c>
+      <c r="E931" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+      <c r="F931" t="inlineStr">
+        <is>
+          <t>FT</t>
+        </is>
+      </c>
+    </row>
+    <row r="932">
+      <c r="A932">
+        <v>2026</v>
+      </c>
+      <c r="B932" t="inlineStr">
+        <is>
+          <t>Mesnil st père</t>
+        </is>
+      </c>
+      <c r="D932" t="inlineStr">
+        <is>
+          <t>50</t>
+        </is>
+      </c>
+      <c r="E932" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+      <c r="F932" t="inlineStr">
+        <is>
+          <t>FT</t>
+        </is>
+      </c>
+    </row>
+    <row r="933">
+      <c r="A933">
+        <v>2026</v>
+      </c>
+      <c r="B933" t="inlineStr">
+        <is>
+          <t>Mesnil st père</t>
+        </is>
+      </c>
+      <c r="D933" t="inlineStr">
+        <is>
+          <t>70</t>
+        </is>
+      </c>
+      <c r="E933" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+      <c r="F933" t="inlineStr">
+        <is>
+          <t>FT</t>
+        </is>
+      </c>
+    </row>
+    <row r="934">
+      <c r="A934">
+        <v>2026</v>
+      </c>
+      <c r="B934" t="inlineStr">
+        <is>
+          <t>Mesnil st père</t>
+        </is>
+      </c>
+      <c r="D934" t="inlineStr">
+        <is>
+          <t>40</t>
+        </is>
+      </c>
+      <c r="E934" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+      <c r="F934" t="inlineStr">
+        <is>
+          <t>FT</t>
+        </is>
+      </c>
+    </row>
+    <row r="935">
+      <c r="A935">
+        <v>2026</v>
+      </c>
+      <c r="B935" t="inlineStr">
+        <is>
+          <t>Mesnil st père</t>
+        </is>
+      </c>
+      <c r="D935" t="inlineStr">
+        <is>
+          <t>45</t>
+        </is>
+      </c>
+      <c r="E935" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+      <c r="F935" t="inlineStr">
+        <is>
+          <t>FT</t>
+        </is>
+      </c>
+    </row>
+    <row r="936">
+      <c r="A936">
+        <v>2026</v>
+      </c>
+      <c r="B936" t="inlineStr">
+        <is>
+          <t>Mesnil st père</t>
+        </is>
+      </c>
+      <c r="D936" t="inlineStr">
+        <is>
+          <t>52</t>
+        </is>
+      </c>
+      <c r="E936" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+      <c r="F936" t="inlineStr">
+        <is>
+          <t>FT</t>
+        </is>
+      </c>
+    </row>
+    <row r="937">
+      <c r="A937">
+        <v>2026</v>
+      </c>
+      <c r="B937" t="inlineStr">
+        <is>
+          <t>Mesnil st père</t>
+        </is>
+      </c>
+      <c r="D937" t="inlineStr">
+        <is>
+          <t>35</t>
+        </is>
+      </c>
+      <c r="E937" t="inlineStr">
+        <is>
+          <t>5</t>
+        </is>
+      </c>
+      <c r="F937" t="inlineStr">
+        <is>
+          <t>FT</t>
+        </is>
+      </c>
+      <c r="J937" t="inlineStr">
+        <is>
+          <t>Oui</t>
+        </is>
+      </c>
+    </row>
+    <row r="938">
+      <c r="A938">
+        <v>2026</v>
+      </c>
+      <c r="B938" t="inlineStr">
+        <is>
+          <t>Mesnil st père</t>
+        </is>
+      </c>
+      <c r="D938" t="inlineStr">
+        <is>
+          <t>30</t>
+        </is>
+      </c>
+      <c r="E938" t="inlineStr">
+        <is>
+          <t>5</t>
+        </is>
+      </c>
+      <c r="F938" t="inlineStr">
+        <is>
+          <t>FT</t>
+        </is>
+      </c>
+    </row>
+    <row r="939">
+      <c r="A939">
+        <v>2026</v>
+      </c>
+      <c r="B939" t="inlineStr">
+        <is>
+          <t>Mesnil st père</t>
+        </is>
+      </c>
+      <c r="D939" t="inlineStr">
+        <is>
+          <t>25</t>
+        </is>
+      </c>
+      <c r="E939" t="inlineStr">
+        <is>
+          <t>10</t>
+        </is>
+      </c>
+      <c r="F939" t="inlineStr">
+        <is>
+          <t>FT</t>
+        </is>
+      </c>
+    </row>
+    <row r="940">
+      <c r="A940">
+        <v>2026</v>
+      </c>
+      <c r="B940" t="inlineStr">
+        <is>
+          <t>Mesnil st père</t>
+        </is>
+      </c>
+      <c r="D940" t="inlineStr">
+        <is>
+          <t>30</t>
+        </is>
+      </c>
+      <c r="E940" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+      <c r="F940" t="inlineStr">
+        <is>
+          <t>FT</t>
+        </is>
+      </c>
+    </row>
+    <row r="941">
+      <c r="A941">
+        <v>2026</v>
+      </c>
+      <c r="B941" t="inlineStr">
+        <is>
+          <t>Mesnil st père</t>
+        </is>
+      </c>
+      <c r="D941" t="inlineStr">
+        <is>
+          <t>50</t>
+        </is>
+      </c>
+      <c r="E941" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+      <c r="F941" t="inlineStr">
+        <is>
+          <t>FT</t>
+        </is>
+      </c>
+    </row>
+    <row r="942">
+      <c r="A942">
+        <v>2026</v>
+      </c>
+      <c r="B942" t="inlineStr">
+        <is>
+          <t>Mesnil st père 2</t>
+        </is>
+      </c>
+      <c r="D942" t="inlineStr">
+        <is>
+          <t>50</t>
+        </is>
+      </c>
+      <c r="E942" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+      <c r="F942" t="inlineStr">
+        <is>
+          <t>FT</t>
+        </is>
+      </c>
+    </row>
+    <row r="943">
+      <c r="A943">
+        <v>2026</v>
+      </c>
+      <c r="B943" t="inlineStr">
+        <is>
+          <t>Mesnil st père 2</t>
+        </is>
+      </c>
+      <c r="D943" t="inlineStr">
+        <is>
+          <t>30</t>
+        </is>
+      </c>
+      <c r="E943" t="inlineStr">
+        <is>
+          <t>31</t>
+        </is>
+      </c>
+      <c r="F943" t="inlineStr">
+        <is>
+          <t>FT</t>
+        </is>
+      </c>
+    </row>
+    <row r="944">
+      <c r="A944">
+        <v>2026</v>
+      </c>
+      <c r="B944" t="inlineStr">
+        <is>
+          <t>Mesnil st père 2</t>
+        </is>
+      </c>
+      <c r="D944" t="inlineStr">
+        <is>
+          <t>30</t>
+        </is>
+      </c>
+      <c r="E944" t="inlineStr">
+        <is>
+          <t>5</t>
+        </is>
+      </c>
+      <c r="F944" t="inlineStr">
+        <is>
+          <t>FT</t>
+        </is>
+      </c>
+    </row>
+    <row r="945">
+      <c r="A945">
+        <v>2026</v>
+      </c>
+      <c r="B945" t="inlineStr">
+        <is>
+          <t>Mesnil st père 2</t>
+        </is>
+      </c>
+      <c r="D945" t="inlineStr">
+        <is>
+          <t>40</t>
+        </is>
+      </c>
+      <c r="E945" t="inlineStr">
+        <is>
+          <t>30</t>
+        </is>
+      </c>
+      <c r="F945" t="inlineStr">
+        <is>
+          <t>FT</t>
+        </is>
+      </c>
+    </row>
+    <row r="946">
+      <c r="A946">
+        <v>2026</v>
+      </c>
+      <c r="B946" t="inlineStr">
+        <is>
+          <t>Mesnil st père 2</t>
+        </is>
+      </c>
+      <c r="D946" t="inlineStr">
+        <is>
+          <t>70</t>
+        </is>
+      </c>
+      <c r="E946" t="inlineStr">
+        <is>
+          <t>20</t>
+        </is>
+      </c>
+      <c r="F946" t="inlineStr">
+        <is>
+          <t>FT</t>
+        </is>
+      </c>
+    </row>
+    <row r="947">
+      <c r="A947">
+        <v>2026</v>
+      </c>
+      <c r="B947" t="inlineStr">
+        <is>
+          <t>Mesnil st père 2</t>
+        </is>
+      </c>
+      <c r="D947" t="inlineStr">
+        <is>
+          <t>40</t>
+        </is>
+      </c>
+      <c r="E947" t="inlineStr">
+        <is>
+          <t>8</t>
+        </is>
+      </c>
+      <c r="F947" t="inlineStr">
+        <is>
+          <t>FT</t>
+        </is>
+      </c>
+    </row>
+    <row r="948">
+      <c r="A948">
+        <v>2026</v>
+      </c>
+      <c r="B948" t="inlineStr">
+        <is>
+          <t>Mesnil st père 2</t>
+        </is>
+      </c>
+      <c r="D948" t="inlineStr">
+        <is>
+          <t>80</t>
+        </is>
+      </c>
+      <c r="E948" t="inlineStr">
+        <is>
+          <t>4</t>
+        </is>
+      </c>
+      <c r="F948" t="inlineStr">
+        <is>
+          <t>FT</t>
+        </is>
+      </c>
+    </row>
+    <row r="949">
+      <c r="A949">
+        <v>2026</v>
+      </c>
+      <c r="B949" t="inlineStr">
+        <is>
+          <t>Mesnil st père 2</t>
+        </is>
+      </c>
+      <c r="D949" t="inlineStr">
+        <is>
+          <t>75</t>
+        </is>
+      </c>
+      <c r="E949" t="inlineStr">
+        <is>
+          <t>8</t>
+        </is>
+      </c>
+      <c r="F949" t="inlineStr">
+        <is>
+          <t>FT</t>
+        </is>
+      </c>
+    </row>
+    <row r="950">
+      <c r="A950">
+        <v>2026</v>
+      </c>
+      <c r="B950" t="inlineStr">
+        <is>
+          <t>Mesnil st père 2</t>
+        </is>
+      </c>
+      <c r="D950" t="inlineStr">
+        <is>
+          <t>80</t>
+        </is>
+      </c>
+      <c r="E950" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+      <c r="F950" t="inlineStr">
+        <is>
+          <t>FT</t>
+        </is>
+      </c>
+    </row>
+    <row r="951">
+      <c r="A951">
+        <v>2026</v>
+      </c>
+      <c r="B951" t="inlineStr">
+        <is>
+          <t>Mesnil st père 2</t>
+        </is>
+      </c>
+      <c r="D951" t="inlineStr">
+        <is>
+          <t>75</t>
+        </is>
+      </c>
+      <c r="E951" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+      <c r="F951" t="inlineStr">
+        <is>
+          <t>FT</t>
+        </is>
+      </c>
+    </row>
+    <row r="952">
+      <c r="A952">
+        <v>2026</v>
+      </c>
+      <c r="B952" t="inlineStr">
+        <is>
+          <t>Mesnil st père 2</t>
+        </is>
+      </c>
+      <c r="D952" t="inlineStr">
+        <is>
+          <t>45</t>
+        </is>
+      </c>
+      <c r="E952" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+      <c r="F952" t="inlineStr">
+        <is>
+          <t>FT</t>
+        </is>
+      </c>
+    </row>
+    <row r="953">
+      <c r="A953">
+        <v>2026</v>
+      </c>
+      <c r="B953" t="inlineStr">
+        <is>
+          <t>Mesnil st père 2</t>
+        </is>
+      </c>
+      <c r="D953" t="inlineStr">
+        <is>
+          <t>55</t>
+        </is>
+      </c>
+      <c r="E953" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+      <c r="F953" t="inlineStr">
+        <is>
+          <t>FT</t>
         </is>
       </c>
     </row>

</xml_diff>